<commit_message>
Resync online NB edits
</commit_message>
<xml_diff>
--- a/MetadataSync/orch_metadata.xlsx
+++ b/MetadataSync/orch_metadata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paul\OneLake - Microsoft\Wave MDF CentralHub\lh_MetadataFileSync.Lakehouse\Files\MetadataSyncFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub_Repos\MDF_CentralHub\MetadataSync\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25397EB0-759C-4EBE-9A21-1F677A13DE12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A9C3B0-A18A-4FB9-80B8-C9B9CC39FF18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21240" yWindow="-19890" windowWidth="25380" windowHeight="16245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22950" yWindow="-18180" windowWidth="25380" windowHeight="16245" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jobs" sheetId="1" r:id="rId1"/>
@@ -24,10 +24,10 @@
   <definedNames>
     <definedName name="DependencyConditionList">DependencyCondition!$A$2:$A$1000</definedName>
     <definedName name="JobNameList">Jobs!$A$2:$A$1000</definedName>
-    <definedName name="ObjectNameList">ObjectIDs!$B$2:$B$998</definedName>
+    <definedName name="ObjectNameList">ObjectIDs!$B$2:$B$999</definedName>
     <definedName name="TaskNameList">Tasks!$A$2:$A$1000</definedName>
     <definedName name="TaskTypeList">TaskType!$A$2:$A$1000</definedName>
-    <definedName name="WorkspaceNameList">ObjectIDs!$A$2:$A$998</definedName>
+    <definedName name="WorkspaceNameList">ObjectIDs!$A$2:$A$999</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -730,7 +730,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="99">
   <si>
     <t>JobName</t>
   </si>
@@ -1012,13 +1012,33 @@
   </si>
   <si>
     <t>Append</t>
+  </si>
+  <si>
+    <t>CopyBronze_WeatherGovDailyForecast</t>
+  </si>
+  <si>
+    <t>nb_WeatherGovApi_ToLakehouse</t>
+  </si>
+  <si>
+    <t>{"latitude": 39.7456, "longitude": -94.6238, ' +
+    '"userAgent": "MDF_CentralHub-demo (REPLACE_ME@yourdomain.example)", ' +
+    '"destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", ' +
+    '"destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0", ' +
+    '"destSchema": "dbo", "destTable": "WeatherGovDailyForecast", ' +
+    '"updateOption": "Append"}</t>
+  </si>
+  <si>
+    <t>Weather</t>
+  </si>
+  <si>
+    <t>PLACEHOLDER</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1038,6 +1058,11 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Cascadia Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1102,7 +1127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1130,6 +1155,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1172,8 +1203,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblTasks" displayName="tblTasks" ref="A1:O28">
-  <autoFilter ref="A1:O28" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblTasks" displayName="tblTasks" ref="A1:O29">
+  <autoFilter ref="A1:O29" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="TaskName"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Include"/>
@@ -1241,8 +1272,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblObjectIDs" displayName="tblObjectIDs" ref="A1:D2">
-  <autoFilter ref="A1:D2" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblObjectIDs" displayName="tblObjectIDs" ref="A1:D3">
+  <autoFilter ref="A1:D3" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="WorkspaceName"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="ObjectName"/>
@@ -1660,13 +1691,13 @@
   <sheetPr>
     <tabColor rgb="FF548235"/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="43.08984375" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="5" max="5" width="20.1796875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="9" width="26" customWidth="1"/>
@@ -2908,6 +2939,50 @@
         <v>25</v>
       </c>
       <c r="O28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>94</v>
+      </c>
+      <c r="B29" t="b">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="E29" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29">
+        <v>1800</v>
+      </c>
+      <c r="G29">
+        <v>1</v>
+      </c>
+      <c r="H29">
+        <v>30</v>
+      </c>
+      <c r="I29" t="s">
+        <v>93</v>
+      </c>
+      <c r="J29" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="L29" t="s">
+        <v>23</v>
+      </c>
+      <c r="M29" t="s">
+        <v>97</v>
+      </c>
+      <c r="N29" t="s">
+        <v>25</v>
+      </c>
+      <c r="O29">
         <v>1</v>
       </c>
     </row>
@@ -2925,7 +3000,7 @@
     <dataValidation type="list" allowBlank="1" sqref="E2:E1000" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>WorkspaceNameList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D1000" xr:uid="{00000000-0002-0000-0100-000004000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D28 D30:D1000" xr:uid="{00000000-0002-0000-0100-000004000000}">
       <formula1>ObjectNameList</formula1>
     </dataValidation>
   </dataValidations>
@@ -3091,12 +3166,12 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="1" max="1" width="20.1796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="61.7265625" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="3" max="3" width="55.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3125,6 +3200,20 @@
         <v>88</v>
       </c>
       <c r="D2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D3" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added notebook to update parallel batch count
</commit_message>
<xml_diff>
--- a/MetadataSync/orch_metadata.xlsx
+++ b/MetadataSync/orch_metadata.xlsx
@@ -1248,7 +1248,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimAccount"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimAccount", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimChannel"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimChannel", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimCurrency"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimCurrency", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimCustomer"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimCustomer", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimDate"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimDate", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimEmployee"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimEmployee", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimEntity"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimEntity", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimGeography"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimGeography", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimMachine"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimMachine", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimOutage"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimOutage", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimProduct"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimProduct", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimProductCategory"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimProductCategory", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimProductSubcategory"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimProductSubcategory", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimPromotion"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimPromotion", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimSalesTerritory"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimSalesTerritory", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimScenario"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimScenario", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "DimStore"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "DimStore", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "FactExchangeRate"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "FactExchangeRate", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "FactInventory"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "FactInventory", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "FactITMachine"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "FactITMachine", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "FactITSLA"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "FactITSLA", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "FactOnlineSales"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "FactOnlineSales", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2612,7 +2612,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "FactSales"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "FactSales", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "FactSalesQuota"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "FactSalesQuota", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "FactSalesSmall"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "FactSalesSmall", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "FactStrategyPlan"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "FactStrategyPlan", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>{"sourceSchema": "dbo", "sourceTable": "YearList"}</t>
+          <t>{"sourceSchema": "dbo", "sourceTable": "YearList", "destWorkspaceId": "947d3136-33ac-458a-be73-ac7dc38afaa5", "destLakehouseId": "649b7795-2e22-4627-8b25-9749a6f492f0"}</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -3170,7 +3170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3245,8 +3245,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
-    <row r="5"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>